<commit_message>
Add ghost prefab and addressable loading
Introduce a Ghost prefab and register it as an Addressable. Add prefab_path to ghosttable.json and regenerate GhostConfig to include PrefabPath. Update EnemyController to instantiate the ghost prefab via Addressables on Bind and release the instance on UnBind (also import Addressables namespace). Add GhostEnum id to EnemyData. Minor scene cleanup (remove Visual child) and update AddressableAssetSettings and source ghost.xlsx.
</commit_message>
<xml_diff>
--- a/Configs/source/Datas/ghost.xlsx
+++ b/Configs/source/Datas/ghost.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t>##var</t>
   </si>
@@ -38,6 +38,9 @@
     <t>desc</t>
   </si>
   <si>
+    <t>prefab_path</t>
+  </si>
+  <si>
     <t>##type</t>
   </si>
   <si>
@@ -60,6 +63,9 @@
   </si>
   <si>
     <t>我是水鬼</t>
+  </si>
+  <si>
+    <t>Ghost/死水鬼.prefab</t>
   </si>
   <si>
     <t>拔舌鬼</t>
@@ -1059,18 +1065,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C23"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="2"/>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="3"/>
   <cols>
     <col min="2" max="2" width="32.8928571428571" customWidth="1"/>
     <col min="3" max="3" width="20.9732142857143" customWidth="1"/>
-    <col min="4" max="4" width="15.1696428571429" customWidth="1"/>
+    <col min="4" max="4" width="19.9464285714286" customWidth="1"/>
     <col min="5" max="5" width="11.6071428571429" customWidth="1"/>
     <col min="6" max="6" width="10.4196428571429" customWidth="1"/>
     <col min="7" max="7" width="17.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:3">
+    <row r="1" s="1" customFormat="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1080,44 +1086,56 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" s="2" customFormat="1" spans="1:3">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" s="2" customFormat="1" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="3" s="3" customFormat="1" spans="1:1">
       <c r="A3" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="1" spans="1:3">
       <c r="A4" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="2:3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4">
       <c r="B5" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="2:3">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4">
       <c r="B6" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>